<commit_message>
Completado dual stack (Parte 2)
</commit_message>
<xml_diff>
--- a/Proyecto 2 - Telemática.xlsx
+++ b/Proyecto 2 - Telemática.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Universidad EAFIT - Ing. de Sistemas\Telemática\proyecto 2\Internet_taller_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFFA6752-8CC9-40D1-AB4E-62F69B76D0E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D118F74-645E-4A1D-BE12-4AF129DD75B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B8D94E8E-8F11-406F-922C-1410950A5C17}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B8D94E8E-8F11-406F-922C-1410950A5C17}"/>
   </bookViews>
   <sheets>
     <sheet name="IPv4" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="127">
   <si>
     <t>Subred</t>
   </si>
@@ -48,15 +48,6 @@
     <t>Hosts</t>
   </si>
   <si>
-    <t>Red base</t>
-  </si>
-  <si>
-    <t>Prefijo</t>
-  </si>
-  <si>
-    <t>Máscara</t>
-  </si>
-  <si>
     <t>Id de Red</t>
   </si>
   <si>
@@ -292,13 +283,286 @@
   </si>
   <si>
     <t>10.10.6.255</t>
+  </si>
+  <si>
+    <t>Prefijo IPv6</t>
+  </si>
+  <si>
+    <t>Dispositivo</t>
+  </si>
+  <si>
+    <t>CLOUD</t>
+  </si>
+  <si>
+    <t>IP Dispositivo</t>
+  </si>
+  <si>
+    <t>2001:DB8:1::/64</t>
+  </si>
+  <si>
+    <t>2001:DB8:2::/64</t>
+  </si>
+  <si>
+    <t>2001:DB8:3::/64</t>
+  </si>
+  <si>
+    <t>2001:DB8:4::/64</t>
+  </si>
+  <si>
+    <t>2001:DB8:5::/64</t>
+  </si>
+  <si>
+    <t>2001:DB8:1::1</t>
+  </si>
+  <si>
+    <t>2001:DB8:2::1</t>
+  </si>
+  <si>
+    <t>2001:DB8:6::/64</t>
+  </si>
+  <si>
+    <t>2001:DB8:3::1</t>
+  </si>
+  <si>
+    <t>2001:DB8:4::1</t>
+  </si>
+  <si>
+    <t>2001:DB8:5::1</t>
+  </si>
+  <si>
+    <t>2001:DB8:6::1</t>
+  </si>
+  <si>
+    <t>PC1</t>
+  </si>
+  <si>
+    <t>PC0</t>
+  </si>
+  <si>
+    <t>SW_VLAN</t>
+  </si>
+  <si>
+    <t>Server2</t>
+  </si>
+  <si>
+    <t>PC2</t>
+  </si>
+  <si>
+    <t>Server1</t>
+  </si>
+  <si>
+    <t>2001:DB8:7::1</t>
+  </si>
+  <si>
+    <t>2001:DB8:8::1</t>
+  </si>
+  <si>
+    <t>2001:DB8:8::/64</t>
+  </si>
+  <si>
+    <t>2001:DB8:7::/64</t>
+  </si>
+  <si>
+    <t>2001:DB8:A::/64</t>
+  </si>
+  <si>
+    <t>2001:DB8:B::/64</t>
+  </si>
+  <si>
+    <t>2001:DB8:C::/64</t>
+  </si>
+  <si>
+    <t>Laptop0</t>
+  </si>
+  <si>
+    <t>2001:DB8:8::2</t>
+  </si>
+  <si>
+    <t>2001:DB8:7::10</t>
+  </si>
+  <si>
+    <t>2001:DB8:3::2</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Router CENTRAL </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>↔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Router LONDON</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Router LONDON </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>↔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Router NEW_YORK</t>
+    </r>
+  </si>
+  <si>
+    <t>CENTRAL: 2001:DB8:A::1    |    LONDON: 2001:DB8:A::2</t>
+  </si>
+  <si>
+    <t>LONDON: 2001:DB8:B::1    |    NEW_YORK: 2001:DB8:B::2</t>
+  </si>
+  <si>
+    <t>NEW_YORK: 2001:DB8:C::1    |    TOKYO: 2001:DB8:C::2</t>
+  </si>
+  <si>
+    <t>2001:DB8:1::10</t>
+  </si>
+  <si>
+    <t>2001:DB8:2::10</t>
+  </si>
+  <si>
+    <t>2001:DB8:4::10</t>
+  </si>
+  <si>
+    <t>2001:DB8:5::10</t>
+  </si>
+  <si>
+    <t>2001:DB8:6::10</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Router NEW_YORK </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>↔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Router TOKYO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Observación:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> VLAN100 pertenece únicamente al switch VLAN (capa 2): </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SE EXCLUYE</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Observación:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Red del router inalámbrico:                    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SE EXCLUYE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -307,15 +571,35 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0" tint="-0.14999847407452621"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -325,6 +609,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -393,12 +695,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -410,21 +724,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -760,7 +1074,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47DA42B5-A694-4E9B-8B1B-E8026BE85A3B}">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="25.77734375" customWidth="1"/>
@@ -772,347 +1086,346 @@
     <col min="9" max="9" width="43.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="8" t="s">
+    <row r="1" spans="1:9" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="F1" s="8" t="s">
+      <c r="I1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="8" t="s">
+    </row>
+    <row r="2" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>10</v>
-      </c>
       <c r="B2" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C2" s="2">
         <v>730</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="H2" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="8"/>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C3" s="2">
         <v>350</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="H3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:9" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2">
+        <v>80</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="1" t="s">
+    </row>
+    <row r="6" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9"/>
+      <c r="B6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2">
+        <v>38</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="8"/>
+      <c r="B7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="2">
+        <v>25</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="2">
-        <v>80</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="K4" s="10"/>
-    </row>
-    <row r="5" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="1" t="s">
+      <c r="C8" s="2">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9"/>
+      <c r="B9" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="C5" s="2">
-        <v>38</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4"/>
-      <c r="B6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="2">
-        <v>25</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="2">
-        <v>4</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="2">
-        <v>2</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4"/>
-      <c r="B9" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="C9" s="2">
         <v>2</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="8"/>
+      <c r="B10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="I10" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="2">
+        <v>100</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="2">
-        <v>100</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="I11" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="2">
+        <v>3</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I12" s="2" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="2">
-        <v>3</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1120,42 +1433,263 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B94C32C6-396E-4BF8-BB58-C57D56B7052D}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="22.88671875" customWidth="1"/>
+    <col min="4" max="4" width="48.77734375" customWidth="1"/>
+    <col min="5" max="5" width="33" customWidth="1"/>
+    <col min="6" max="6" width="23.109375" customWidth="1"/>
+    <col min="8" max="8" width="15.44140625" customWidth="1"/>
+    <col min="9" max="9" width="14.5546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="C1" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="E1" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="B2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="11"/>
+      <c r="B3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="11"/>
+      <c r="B4" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+    </row>
+    <row r="5" spans="1:10" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="11"/>
+      <c r="B6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="11"/>
+      <c r="B7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
         <v>9</v>
       </c>
+      <c r="B8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" s="12"/>
+    </row>
+    <row r="9" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="11"/>
+      <c r="B9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="11"/>
+      <c r="B10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="64.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+    </row>
+    <row r="12" spans="1:10" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>111</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="H4:J4"/>
+  </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>